<commit_message>
docs(example): regenerate the quotation export with its new columns
make examples stopped at the first 204 (send), since its json helper
parsed every answer as JSON. With that fixed, only the quotation list
export is committed; the other regenerated files were left out to keep
this change to the export it is about.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/quotation-export.xlsx
+++ b/docs/example/quotation-export.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>No. Quotation</t>
   </si>
@@ -28,25 +28,40 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Subtotal</t>
+    <t>Total Produk</t>
   </si>
   <si>
     <t>Diskon</t>
   </si>
   <si>
+    <t>Pengiriman</t>
+  </si>
+  <si>
+    <t>Sub Total</t>
+  </si>
+  <si>
+    <t>PPN</t>
+  </si>
+  <si>
+    <t>Nilai PPN</t>
+  </si>
+  <si>
     <t>Grand Total</t>
   </si>
   <si>
     <t>Q-00001/GNS/X/2026</t>
   </si>
   <si>
-    <t>2026-10-10</t>
+    <t>2026-10-11</t>
   </si>
   <si>
     <t>PT Samudra Contoh Nusantara</t>
   </si>
   <si>
     <t>Disetujui</t>
+  </si>
+  <si>
+    <t>12%</t>
   </si>
 </sst>
 </file>
@@ -388,27 +403,51 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E2" s="2">
-        <v>17622000</v>
+        <v>17760000</v>
       </c>
       <c r="F2" s="2">
         <v>888000</v>
       </c>
       <c r="G2" s="2">
+        <v>750000</v>
+      </c>
+      <c r="H2" s="2">
+        <v>17622000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1938420</v>
+      </c>
+      <c r="K2" s="2">
         <v>19560420</v>
       </c>
     </row>

</xml_diff>